<commit_message>
Add Product 28 Juli 26
</commit_message>
<xml_diff>
--- a/Report_SignUp.xlsx
+++ b/Report_SignUp.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="344">
   <si>
     <t>No</t>
   </si>
@@ -889,6 +889,168 @@
   </si>
   <si>
     <t>087667495127</t>
+  </si>
+  <si>
+    <t>2026-07-27 22:30:30</t>
+  </si>
+  <si>
+    <t>Ramadhany7814</t>
+  </si>
+  <si>
+    <t>ramatest.7814@gmail.com</t>
+  </si>
+  <si>
+    <t>rama7814</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>1984</t>
+  </si>
+  <si>
+    <t>testrama7814</t>
+  </si>
+  <si>
+    <t>testnur7814</t>
+  </si>
+  <si>
+    <t>1204</t>
+  </si>
+  <si>
+    <t>087721429456</t>
+  </si>
+  <si>
+    <t>2026-07-27 23:25:55</t>
+  </si>
+  <si>
+    <t>Ramadhany2946</t>
+  </si>
+  <si>
+    <t>ramatest.2946@gmail.com</t>
+  </si>
+  <si>
+    <t>rama2946</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>testrama2946</t>
+  </si>
+  <si>
+    <t>testnur2946</t>
+  </si>
+  <si>
+    <t>NurSejahtera95</t>
+  </si>
+  <si>
+    <t>Jalan Kampung selatan95</t>
+  </si>
+  <si>
+    <t>Kemayoran Lama, Jakarta, 95</t>
+  </si>
+  <si>
+    <t>Jakarta95</t>
+  </si>
+  <si>
+    <t>Jakarta Pusat95</t>
+  </si>
+  <si>
+    <t>1103</t>
+  </si>
+  <si>
+    <t>087776906019</t>
+  </si>
+  <si>
+    <t>2026-07-27 23:39:04</t>
+  </si>
+  <si>
+    <t>Ramadhany2312</t>
+  </si>
+  <si>
+    <t>ramatest.2312@gmail.com</t>
+  </si>
+  <si>
+    <t>rama2312</t>
+  </si>
+  <si>
+    <t>2008</t>
+  </si>
+  <si>
+    <t>testrama2312</t>
+  </si>
+  <si>
+    <t>testnur2312</t>
+  </si>
+  <si>
+    <t>NurSejahtera93</t>
+  </si>
+  <si>
+    <t>Jalan Kampung selatan93</t>
+  </si>
+  <si>
+    <t>Kemayoran Lama, Jakarta, 93</t>
+  </si>
+  <si>
+    <t>Jakarta93</t>
+  </si>
+  <si>
+    <t>Jakarta Pusat93</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>087844405135</t>
+  </si>
+  <si>
+    <t>2026-07-28 15:30:38</t>
+  </si>
+  <si>
+    <t>Ramadhany3533</t>
+  </si>
+  <si>
+    <t>ramatest.3533@gmail.com</t>
+  </si>
+  <si>
+    <t>rama3533</t>
+  </si>
+  <si>
+    <t>1993</t>
+  </si>
+  <si>
+    <t>testrama3533</t>
+  </si>
+  <si>
+    <t>testnur3533</t>
+  </si>
+  <si>
+    <t>NurSejahtera63</t>
+  </si>
+  <si>
+    <t>Jalan Kampung selatan63</t>
+  </si>
+  <si>
+    <t>Kemayoran Lama, Jakarta, 63</t>
+  </si>
+  <si>
+    <t>Jakarta63</t>
+  </si>
+  <si>
+    <t>Jakarta Pusat63</t>
+  </si>
+  <si>
+    <t>11064</t>
+  </si>
+  <si>
+    <t>087967041719</t>
   </si>
 </sst>
 </file>
@@ -1259,7 +1421,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="12.0" collapsed="true"/>
@@ -2575,6 +2737,278 @@
         <v>41</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19.0</v>
+      </c>
+      <c r="B20" t="s">
+        <v>290</v>
+      </c>
+      <c r="C20" t="s">
+        <v>291</v>
+      </c>
+      <c r="D20" t="s">
+        <v>292</v>
+      </c>
+      <c r="E20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" t="s">
+        <v>293</v>
+      </c>
+      <c r="G20" t="s">
+        <v>294</v>
+      </c>
+      <c r="H20" t="s">
+        <v>295</v>
+      </c>
+      <c r="I20" t="s">
+        <v>296</v>
+      </c>
+      <c r="J20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K20" t="s">
+        <v>30</v>
+      </c>
+      <c r="L20" t="s">
+        <v>297</v>
+      </c>
+      <c r="M20" t="s">
+        <v>298</v>
+      </c>
+      <c r="N20" t="s">
+        <v>244</v>
+      </c>
+      <c r="O20" t="s">
+        <v>245</v>
+      </c>
+      <c r="P20" t="s">
+        <v>246</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>109</v>
+      </c>
+      <c r="R20" t="s">
+        <v>247</v>
+      </c>
+      <c r="S20" t="s">
+        <v>248</v>
+      </c>
+      <c r="T20" t="s">
+        <v>299</v>
+      </c>
+      <c r="U20" t="s">
+        <v>300</v>
+      </c>
+      <c r="V20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="B21" t="s">
+        <v>301</v>
+      </c>
+      <c r="C21" t="s">
+        <v>302</v>
+      </c>
+      <c r="D21" t="s">
+        <v>303</v>
+      </c>
+      <c r="E21" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21" t="s">
+        <v>304</v>
+      </c>
+      <c r="G21" t="s">
+        <v>305</v>
+      </c>
+      <c r="H21" t="s">
+        <v>306</v>
+      </c>
+      <c r="I21" t="s">
+        <v>255</v>
+      </c>
+      <c r="J21" t="s">
+        <v>30</v>
+      </c>
+      <c r="K21" t="s">
+        <v>30</v>
+      </c>
+      <c r="L21" t="s">
+        <v>307</v>
+      </c>
+      <c r="M21" t="s">
+        <v>308</v>
+      </c>
+      <c r="N21" t="s">
+        <v>309</v>
+      </c>
+      <c r="O21" t="s">
+        <v>310</v>
+      </c>
+      <c r="P21" t="s">
+        <v>311</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>64</v>
+      </c>
+      <c r="R21" t="s">
+        <v>312</v>
+      </c>
+      <c r="S21" t="s">
+        <v>313</v>
+      </c>
+      <c r="T21" t="s">
+        <v>314</v>
+      </c>
+      <c r="U21" t="s">
+        <v>315</v>
+      </c>
+      <c r="V21" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21.0</v>
+      </c>
+      <c r="B22" t="s">
+        <v>316</v>
+      </c>
+      <c r="C22" t="s">
+        <v>317</v>
+      </c>
+      <c r="D22" t="s">
+        <v>318</v>
+      </c>
+      <c r="E22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22" t="s">
+        <v>319</v>
+      </c>
+      <c r="G22" t="s">
+        <v>28</v>
+      </c>
+      <c r="H22" t="s">
+        <v>64</v>
+      </c>
+      <c r="I22" t="s">
+        <v>320</v>
+      </c>
+      <c r="J22" t="s">
+        <v>30</v>
+      </c>
+      <c r="K22" t="s">
+        <v>30</v>
+      </c>
+      <c r="L22" t="s">
+        <v>321</v>
+      </c>
+      <c r="M22" t="s">
+        <v>322</v>
+      </c>
+      <c r="N22" t="s">
+        <v>323</v>
+      </c>
+      <c r="O22" t="s">
+        <v>324</v>
+      </c>
+      <c r="P22" t="s">
+        <v>325</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>36</v>
+      </c>
+      <c r="R22" t="s">
+        <v>326</v>
+      </c>
+      <c r="S22" t="s">
+        <v>327</v>
+      </c>
+      <c r="T22" t="s">
+        <v>328</v>
+      </c>
+      <c r="U22" t="s">
+        <v>329</v>
+      </c>
+      <c r="V22" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22.0</v>
+      </c>
+      <c r="B23" t="s">
+        <v>330</v>
+      </c>
+      <c r="C23" t="s">
+        <v>331</v>
+      </c>
+      <c r="D23" t="s">
+        <v>332</v>
+      </c>
+      <c r="E23" t="s">
+        <v>25</v>
+      </c>
+      <c r="F23" t="s">
+        <v>333</v>
+      </c>
+      <c r="G23" t="s">
+        <v>64</v>
+      </c>
+      <c r="H23" t="s">
+        <v>63</v>
+      </c>
+      <c r="I23" t="s">
+        <v>334</v>
+      </c>
+      <c r="J23" t="s">
+        <v>30</v>
+      </c>
+      <c r="K23" t="s">
+        <v>30</v>
+      </c>
+      <c r="L23" t="s">
+        <v>335</v>
+      </c>
+      <c r="M23" t="s">
+        <v>336</v>
+      </c>
+      <c r="N23" t="s">
+        <v>337</v>
+      </c>
+      <c r="O23" t="s">
+        <v>338</v>
+      </c>
+      <c r="P23" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>109</v>
+      </c>
+      <c r="R23" t="s">
+        <v>340</v>
+      </c>
+      <c r="S23" t="s">
+        <v>341</v>
+      </c>
+      <c r="T23" t="s">
+        <v>342</v>
+      </c>
+      <c r="U23" t="s">
+        <v>343</v>
+      </c>
+      <c r="V23" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>